<commit_message>
docs: atualiza arquivos de categorização e seeds
- Categorias.xlsx atualizado
- Seeds de lançados e não lançados revistos
- Documentação de categorização atualizada
- Arquivos de referência sincronizados

Co-Authored-By: Claude Haiku 4.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CATEGORIAS.xlsx
+++ b/CATEGORIAS.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\guilherme.frade\Desktop\Backup Guilherme\BACKUP - Guilherme\BACKUP - Guilherme\Automacao_python\sistema_de_ouvidoria\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{24E9B1C3-6D53-4286-AB85-701D352BBA1F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6A3271B-EBBC-4A87-9DBB-8066774E2DC2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{4145407C-2983-4B65-84D6-7DCFF87F1F3F}"/>
   </bookViews>
@@ -68,9 +68,6 @@
     <t>COBRANÇA OU TARIFA</t>
   </si>
   <si>
-    <t>INFORMAÇÕES SOBRE O SERVIÇO</t>
-  </si>
-  <si>
     <t>ATRASO / ADIANTAMENTO DE VEÍCULO</t>
   </si>
   <si>
@@ -147,6 +144,9 @@
   </si>
   <si>
     <t>REPLICA</t>
+  </si>
+  <si>
+    <t>FALHA NA COMUNICAÇÃO/DIVULGAÇÃO</t>
   </si>
 </sst>
 </file>
@@ -650,7 +650,7 @@
     </row>
     <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="3" t="s">
-        <v>10</v>
+        <v>36</v>
       </c>
       <c r="B9" s="3" t="s">
         <v>3</v>
@@ -658,7 +658,7 @@
     </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>3</v>
@@ -666,7 +666,7 @@
     </row>
     <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="B11" s="3" t="s">
         <v>3</v>
@@ -674,7 +674,7 @@
     </row>
     <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>3</v>
@@ -682,7 +682,7 @@
     </row>
     <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B13" s="3" t="s">
         <v>3</v>
@@ -690,7 +690,7 @@
     </row>
     <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="2" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>3</v>
@@ -698,7 +698,7 @@
     </row>
     <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="3" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>3</v>
@@ -706,7 +706,7 @@
     </row>
     <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>3</v>
@@ -714,7 +714,7 @@
     </row>
     <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B17" s="3" t="s">
         <v>3</v>
@@ -722,7 +722,7 @@
     </row>
     <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>3</v>
@@ -730,7 +730,7 @@
     </row>
     <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>3</v>
@@ -738,7 +738,7 @@
     </row>
     <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>3</v>
@@ -746,7 +746,7 @@
     </row>
     <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="3" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B21" s="3" t="s">
         <v>3</v>
@@ -754,7 +754,7 @@
     </row>
     <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>3</v>
@@ -762,7 +762,7 @@
     </row>
     <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="B23" s="4" t="s">
         <v>3</v>
@@ -770,7 +770,7 @@
     </row>
     <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>3</v>
@@ -778,7 +778,7 @@
     </row>
     <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="4" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="B25" s="4" t="s">
         <v>3</v>
@@ -786,50 +786,50 @@
     </row>
     <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
+        <v>26</v>
+      </c>
+      <c r="B26" s="5" t="s">
         <v>27</v>
-      </c>
-      <c r="B26" s="5" t="s">
-        <v>28</v>
       </c>
     </row>
     <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="B27" s="4" t="s">
         <v>29</v>
-      </c>
-      <c r="B27" s="4" t="s">
-        <v>30</v>
       </c>
     </row>
     <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="B28" s="5" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="B29" s="4" t="s">
         <v>32</v>
-      </c>
-      <c r="B29" s="4" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B30" s="5" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="B31" s="6" t="s">
         <v>35</v>
-      </c>
-      <c r="B31" s="6" t="s">
-        <v>36</v>
       </c>
     </row>
   </sheetData>

</xml_diff>